<commit_message>
feat(F-NAR-019): ATOM-AUT.ROU.001-03 Le pain chaud de Nino
</commit_message>
<xml_diff>
--- a/stories/arbres/ATOM-AUT.ROU.001-03.xlsx
+++ b/stories/arbres/ATOM-AUT.ROU.001-03.xlsx
@@ -841,7 +841,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Nino sent le pain chaud et veut descendre tout de suite. Papa l'attend à la marche. Une chose puis la suivante, il mord la croûte tiède.</t>
+          <t>En bas, un plat se pose. Toc. Sur la première marche, un éclat de marche brille. Nino veut le pain chaud maintenant. Il court en pyjama : le pied glisse. Il refuse de foncer, met le pull jaune, ramasse la chaussette. L'éclat de marche guide. Sur la croûte, l'éclat garde une trace.</t>
         </is>
       </c>
     </row>
@@ -1184,17 +1184,17 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>Une odeur de pain monte l'escalier. Ça sent le beurre. Ça sent la croûte dorée. Une petite vapeur grimpe, toute blanche. Les marches de bois sont lisses. La rampe est ronde sous la main. En bas, un plat se pose. Ça fait un petit bruit. Nino, tu sens le pain ? Oui, maman. C'est chaud. Il est sur la planche. En ce moment, Nino est dans son lit. L'oreiller est plat. Le drap sent le sommeil. Je veux le pain. Nino pose un pied par terre. Il va vers la première marche. Il est encore en pyjama. Le pain t'attend, Nino. D'abord le pull. Une chose, puis la suivante. Nino s'arrête. L'odeur est encore là. Elle est douce, très douce. Il part, le pain ? Non. Il reste au chaud. On se lève ? Oui. Nino revient vers le lit. Ses pieds touchent le tapis. Le pull jaune, d'abord.</t>
+          <t>En bas, un plat se pose. Toc. Une vapeur grimpe l'escalier. Elle sent le beurre. Ça sent la croûte dorée. Sur la première marche, un éclat de marche brille. Il est blanc, maman. C'est la vapeur du pain. L'éclat de marche tient comme une petite lune. Les marches de bois sont lisses. La rampe est ronde sous la main. Un carré de soleil touche le bois. La chambre sent le pain, tiède. Nino, tu sens le pain ? Oui, papa. Je le veux, maintenant. Il est sur la planche, en bas. Le pull jaune attend près du lit. En ce moment, Nino est dans son lit. L'oreiller est plat. Le drap sent le sommeil. Plus tard, le pull. Nino pose un pied par terre. Le tapis est chaud sous les orteils. Il court vers l'escalier, en pyjama. Sa main rate la rampe. Son pied glisse sur l'éclat de marche. Oh. Il s'assoit d'un coup, sur la marche. Le sourire de Nino disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Le pain part ? Non. Il reste au chaud. Nino veut redescendre d'un seul élan. Ses épaules tombent un peu. Ça serre, dans son ventre. Papa se baisse à sa hauteur. Tu regardes la marche ?</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>Une odeur de pain monte l'escalier. Ça sent le beurre. Ça sent la croûte dorée. Une petite vapeur grimpe, toute blanche. Les marches de bois sont lisses. La rampe est ronde sous la main. En bas, un plat se pose. Ça fait un petit bruit. Nino, tu sens le pain ? Oui, maman. C'est chaud. Il est sur la planche. En ce moment, Nino est dans son lit. L'oreiller est plat. Le drap sent le sommeil. Je veux le pain. Nino pose un pied par terre. Il va vers la première marche. Il est encore en pyjama. Le pain t'attend, Nino. D'abord le pull. Une chose, puis la suivante. Nino s'arrête. L'odeur est encore là. Elle est douce, très douce. Il part, le pain ? Non. Il reste au chaud. On se lève ? Oui. Nino revient vers le lit. Ses pieds touchent le tapis. Le pull jaune, d'abord.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;En bas, un plat se pose. Toc. Une vapeur grimpe l'escalier. Elle sent le beurre. Ça sent la croûte dorée. Sur la première marche, un &lt;emphasis level="moderate"&gt;éclat de marche&lt;/emphasis&gt; brille. Il est blanc, maman. C'est la vapeur du pain. L'éclat de marche tient comme une petite lune. Les marches de bois sont lisses. La rampe est ronde sous la main. Un carré de soleil touche le bois. La chambre sent le pain, tiède. Nino, tu sens le pain ? Oui, papa. Je le veux, maintenant. Il est sur la planche, en bas. Le pull jaune attend près du lit. En ce moment, Nino est dans son lit. L'oreiller est plat. Le drap sent le sommeil. Plus tard, le pull. Nino pose un pied par terre. Le tapis est chaud sous les orteils. Il court vers l'escalier, en pyjama. Sa main rate la rampe. Son pied glisse sur l'éclat de marche. Oh. Il s'assoit d'un coup, sur la marche. Le sourire de Nino disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Le pain part ? Non. Il reste au chaud. Nino veut redescendre d'un seul élan. Ses épaules tombent un peu. Ça serre, dans son ventre. Papa se baisse à sa hauteur. Tu regardes la marche ?&lt;/prosody&gt;&lt;break time="500ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;Le soleil entre. Ilyes ouvre les yeux. Le drap est chaud. Papa dit : c'est le matin. &lt;emphasis&gt;une&lt;/emphasis&gt; étape après l'autre. D'abord, Ilyes se lève. Ses pieds touchent le tapis. Le tapis est doux. Ensuite, Ilyes s'habille. Il met le pull vert. Il met le pantalon. Les chaussettes aussi. Maman dit : maintenant, le déjeuner. Ilyes s'assoit à table. Il mange du pain. Il boit du lait tiède. Papa dit : ensuite, le sac. Ilyes met la gourde dans le sac. Ilyes met le doudou dans le sac. Une étape après l'autre. Ilyes est prêt. Papa dit : une étape après l'autre.&lt;/slow&gt; [pause]</t>
+          <t>En bas, un plat se pose. Toc. Une vapeur grimpe l'escalier. Elle sent le beurre. Ça sent la croûte dorée. Sur la première marche, un &lt;emphasis&gt;éclat de marche&lt;/emphasis&gt; brille. Il est blanc, maman. C'est la vapeur du pain. L'éclat de marche tient comme une petite lune. Les marches de bois sont lisses. La rampe est ronde sous la main. Un carré de soleil touche le bois. La chambre sent le pain, tiède. Nino, tu sens le pain ? Oui, papa. Je le veux, maintenant. Il est sur la planche, en bas. Le pull jaune attend près du lit. En ce moment, Nino est dans son lit. L'oreiller est plat. Le drap sent le sommeil. Plus tard, le pull. Nino pose un pied par terre. Le tapis est chaud sous les orteils. Il court vers l'escalier, en pyjama. Sa main rate la rampe. Son pied glisse sur l'éclat de marche. Oh. Il s'assoit d'un coup, sur la marche. Le sourire de Nino disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Le pain part ? Non. Il reste au chaud. Nino veut redescendre d'un seul élan. Ses épaules tombent un peu. Ça serre, dans son ventre. Papa se baisse à sa hauteur. Tu regardes la marche ? [pause]</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr"/>
@@ -1241,7 +1241,7 @@
         </is>
       </c>
       <c r="Y2" s="2" t="n">
-        <v>118</v>
+        <v>142</v>
       </c>
       <c r="Z2" s="2" t="inlineStr">
         <is>
@@ -1249,10 +1249,10 @@
         </is>
       </c>
       <c r="AA2" s="2" t="n">
-        <v>0.86</v>
+        <v>0.98</v>
       </c>
       <c r="AB2" s="2" t="n">
-        <v>1.22</v>
+        <v>1.12</v>
       </c>
       <c r="AC2" s="2" t="inlineStr">
         <is>
@@ -1275,30 +1275,30 @@
       </c>
       <c r="AH2" s="2" t="inlineStr">
         <is>
-          <t>une</t>
+          <t>éclat de marche</t>
         </is>
       </c>
       <c r="AI2" s="2" t="n">
         <v>0</v>
       </c>
       <c r="AJ2" s="2" t="n">
-        <v>400</v>
+        <v>500</v>
       </c>
       <c r="AK2" s="2" t="n">
-        <v>380</v>
+        <v>260</v>
       </c>
       <c r="AL2" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>warm</t>
         </is>
       </c>
       <c r="AM2" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>storytelling</t>
         </is>
       </c>
       <c r="AN2" s="2" t="n">
-        <v>0.333</v>
+        <v>0.36</v>
       </c>
       <c r="AO2" s="2" t="inlineStr"/>
       <c r="AP2" s="2" t="inlineStr">
@@ -1307,10 +1307,10 @@
         </is>
       </c>
       <c r="AQ2" s="2" t="n">
-        <v>0.86</v>
+        <v>0.98</v>
       </c>
       <c r="AR2" s="2" t="n">
-        <v>0.86</v>
+        <v>0.98</v>
       </c>
       <c r="AS2" s="2" t="n">
         <v>100</v>
@@ -1319,49 +1319,59 @@
         <v>50</v>
       </c>
       <c r="AU2" s="2" t="n">
-        <v>12</v>
-      </c>
-      <c r="AV2" s="2" t="inlineStr"/>
+        <v>8</v>
+      </c>
+      <c r="AV2" s="2" t="inlineStr">
+        <is>
+          <t>arc=installation; intention=émerveiller puis tendre; emotion=impatience puis découragement; intensite=2; destinataire=enfant; sous_texte=il_veut_le_pain_chaud_maintenant; tempo=naturel puis resserré; sourire=léger puis aucun; respiration=ample puis retenue</t>
+        </is>
+      </c>
       <c r="AW2" t="inlineStr">
         <is>
-          <t>narrateur|Une odeur de pain monte l'escalier.
-narrateur|Ça sent le beurre.
+          <t>narrateur|En bas, un plat se pose.
+narrateur|Toc.
+narrateur|Une vapeur grimpe l'escalier.
+narrateur|Elle sent le beurre.
 narrateur|Ça sent la croûte dorée.
-narrateur|Une petite vapeur grimpe, toute blanche.
+narrateur|Sur la première marche, un éclat de marche brille.
+enfant-m|Il est blanc, maman.
+maman|C'est la vapeur du pain.
+narrateur|L'éclat de marche tient comme une petite lune.
 narrateur|Les marches de bois sont lisses.
 narrateur|La rampe est ronde sous la main.
-narrateur|En bas, un plat se pose.
-narrateur|Ça fait un petit bruit.
-maman|Nino, tu sens le pain ?
-enfant-m|Oui, maman.
-enfant-m|C'est chaud.
-papa|Il est sur la planche.
+narrateur|Un carré de soleil touche le bois.
+narrateur|La chambre sent le pain, tiède.
+papa|Nino, tu sens le pain ?
+enfant-m|Oui, papa.
+enfant-m|Je le veux, maintenant.
+papa|Il est sur la planche, en bas.
+narrateur|Le pull jaune attend près du lit.
 narrateur|En ce moment, Nino est dans son lit.
 narrateur|L'oreiller est plat.
 narrateur|Le drap sent le sommeil.
-enfant-m|Je veux le pain.
+enfant-m|Plus tard, le pull.
 narrateur|Nino pose un pied par terre.
-narrateur|Il va vers la première marche.
-narrateur|Il est encore en pyjama.
-papa|Le pain t'attend, Nino.
-papa|D'abord le pull.
-maman|Une chose, puis la suivante.
-narrateur|Nino s'arrête.
-narrateur|L'odeur est encore là.
-narrateur|Elle est douce, très douce.
-enfant-m|Il part, le pain ?
+narrateur|Le tapis est chaud sous les orteils.
+narrateur|Il court vers l'escalier, en pyjama.
+narrateur|Sa main rate la rampe.
+narrateur|Son pied glisse sur l'éclat de marche.
+enfant-m|Oh.
+narrateur|Il s'assoit d'un coup, sur la marche.
+narrateur|Le sourire de Nino disparaît.
+narrateur|Dans sa poitrine, l'envie et l'inquiétude se bousculent.
+enfant-m|Le pain part ?
 maman|Non.
 maman|Il reste au chaud.
-papa|On se lève ?
-enfant-m|Oui.
-narrateur|Nino revient vers le lit.
-narrateur|Ses pieds touchent le tapis.
-papa|Le pull jaune, d'abord.</t>
+narrateur|Nino veut redescendre d'un seul élan.
+narrateur|Ses épaules tombent un peu.
+narrateur|Ça serre, dans son ventre.
+narrateur|Papa se baisse à sa hauteur.
+papa|Tu regardes la marche ?</t>
         </is>
       </c>
       <c r="AX2" t="inlineStr">
         <is>
-          <t>pain</t>
+          <t>pain,vapeur</t>
         </is>
       </c>
     </row>
@@ -1393,12 +1403,12 @@
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>Nino veut le pain. Comment se prépare-t-il ?</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="medium"&gt;Nino veut le &lt;emphasis level="moderate"&gt;pain&lt;/emphasis&gt;. Comment se prépare-t-il ?&lt;/prosody&gt;&lt;break time="700ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;Ilyes se prépare. Comment avance-t-il ?&lt;/slow&gt;</t>
+          <t>&lt;soft&gt;&lt;slow&gt;Nino veut le &lt;emphasis&gt;pain&lt;/emphasis&gt;. Comment se prépare-t-il ?&lt;/slow&gt;&lt;/soft&gt; [pause]</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -1461,7 +1471,7 @@
         </is>
       </c>
       <c r="Y3" s="2" t="n">
-        <v>100</v>
+        <v>120</v>
       </c>
       <c r="Z3" s="2" t="inlineStr">
         <is>
@@ -1469,10 +1479,10 @@
         </is>
       </c>
       <c r="AA3" s="2" t="n">
-        <v>0.8</v>
+        <v>0.86</v>
       </c>
       <c r="AB3" s="2" t="n">
-        <v>1.28</v>
+        <v>1.27</v>
       </c>
       <c r="AC3" s="2" t="inlineStr">
         <is>
@@ -1487,34 +1497,38 @@
       <c r="AE3" s="2" t="inlineStr"/>
       <c r="AF3" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>soft</t>
         </is>
       </c>
       <c r="AG3" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="AH3" s="2" t="inlineStr"/>
+        <v>-2</v>
+      </c>
+      <c r="AH3" s="2" t="inlineStr">
+        <is>
+          <t>pain</t>
+        </is>
+      </c>
       <c r="AI3" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ3" s="2" t="n">
-        <v>250</v>
+        <v>700</v>
       </c>
       <c r="AK3" s="2" t="n">
-        <v>380</v>
+        <v>320</v>
       </c>
       <c r="AL3" s="2" t="inlineStr">
         <is>
-          <t>warm</t>
+          <t>focused</t>
         </is>
       </c>
       <c r="AM3" s="2" t="inlineStr">
         <is>
-          <t>rise</t>
+          <t>rising</t>
         </is>
       </c>
       <c r="AN3" s="2" t="n">
-        <v>0.333</v>
+        <v>0.32</v>
       </c>
       <c r="AO3" s="2" t="inlineStr"/>
       <c r="AP3" s="2" t="inlineStr">
@@ -1523,13 +1537,13 @@
         </is>
       </c>
       <c r="AQ3" s="2" t="n">
-        <v>0.8</v>
+        <v>0.86</v>
       </c>
       <c r="AR3" s="2" t="n">
-        <v>0.8</v>
+        <v>0.86</v>
       </c>
       <c r="AS3" s="2" t="n">
-        <v>100</v>
+        <v>82</v>
       </c>
       <c r="AT3" s="2" t="n">
         <v>50</v>
@@ -1539,7 +1553,7 @@
       </c>
       <c r="AV3" s="2" t="inlineStr">
         <is>
-          <t>question d'écoute, ne change pas le cours</t>
+          <t>arc=indice; intention=faire_deviner; emotion=attention; intensite=1; destinataire=enfant; sous_texte=il_se_prepare_une_chose_apres_l_autre; tempo=suspendu; sourire=aucun; respiration=courte_avant_question</t>
         </is>
       </c>
       <c r="AW3" t="inlineStr">
@@ -1572,17 +1586,17 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Le pull jaune est près du lit. Nino enfile le pull. Le pull est doux sur les bras. C'est fait. Ensuite, les marches. Nino pose la main sur la rampe. Une marche, puis l'autre. Oui, maman. Les marches sentent le bois. La cuisine est chaude. Le pain est sur la planche. La croûte craque un peu. Tu t'assois ? Nino s'assoit à table. Un peu de beurre ? Oui, un peu. Merci, Nino.</t>
+          <t>Nino revient vers le lit. Ses pieds touchent le tapis. Le pull jaune est près du lit. Toi d'abord. Il enfile le pull. Le pull est doux sur les bras. Le pyjama reste en dessous, chaud. C'est fait. Tu vas vers les marches ? Oui, maman. Nino s'arrête devant la première marche. L'éclat de marche brille, petit. Je te vois. Sa main trouve la rampe. La rampe est ronde, un peu froide. Une marche, sous le pied. Puis une autre. Je regarde. Au milieu, une chaussette traîne. Je la pousse. Nino lève le pied, trop vite. Puis il s'arrête. Attends. Nino refuse de foncer. Il ramasse la chaussette. Sous le tissu, l'éclat de marche brille. Comme en haut ! Tu le vois, toi ? Oui, près du bois. Nino glisse la chaussette dans sa main. Il descend, sans sauter. La cuisine est chaude. Le pain est sur la planche. Merci, tu as regardé. Te voilà. Il est chaud.</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Le pull jaune est près du lit. Nino enfile le pull. Le pull est doux sur les bras. C'est fait. Ensuite, les marches. Nino pose la main sur la rampe. Une marche, puis l'autre. Oui, maman. Les marches sentent le bois. La cuisine est chaude. Le pain est sur la planche. La croûte craque un peu. Tu t'assois ? Nino s'assoit à table. Un peu de beurre ? Oui, un peu. Merci, Nino.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Nino revient vers le lit. Ses pieds touchent le tapis. Le pull jaune est près du lit. Toi d'abord. Il enfile le pull. Le pull est doux sur les bras. Le pyjama reste en dessous, chaud. C'est fait. Tu vas vers les marches ? Oui, maman. Nino s'arrête devant la première marche. L'&lt;emphasis level="moderate"&gt;éclat de marche&lt;/emphasis&gt; brille, petit. Je te vois. Sa main trouve la rampe. La rampe est ronde, un peu froide. Une marche, sous le pied. Puis une autre. Je regarde. Au milieu, une chaussette traîne. Je la pousse. Nino lève le pied, trop vite. Puis il s'arrête. Attends. Nino refuse de foncer. Il ramasse la chaussette. Sous le tissu, l'éclat de marche brille. Comme en haut ! Tu le vois, toi ? Oui, près du bois. Nino glisse la chaussette dans sa main. Il descend, sans sauter. La cuisine est chaude. Le pain est sur la planche. Merci, tu as regardé. Te voilà. Il est chaud.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;Ilyes a fait l'étape dite. Se lever. S'habiller. Déje&lt;emphasis&gt;une&lt;/emphasis&gt;r. Le sac. Une étape après l'autre.&lt;/slow&gt; [pause]</t>
+          <t>Nino revient vers le lit. Ses pieds touchent le tapis. Le pull jaune est près du lit. Toi d'abord. Il enfile le pull. Le pull est doux sur les bras. Le pyjama reste en dessous, chaud. C'est fait. Tu vas vers les marches ? Oui, maman. Nino s'arrête devant la première marche. L'&lt;emphasis&gt;éclat de marche&lt;/emphasis&gt; brille, petit. Je te vois. Sa main trouve la rampe. La rampe est ronde, un peu froide. Une marche, sous le pied. Puis une autre. Je regarde. Au milieu, une chaussette traîne. Je la pousse. Nino lève le pied, trop vite. Puis il s'arrête. Attends. Nino refuse de foncer. Il ramasse la chaussette. Sous le tissu, l'éclat de marche brille. Comme en haut ! Tu le vois, toi ? Oui, près du bois. Nino glisse la chaussette dans sa main. Il descend, sans sauter. La cuisine est chaude. Le pain est sur la planche. Merci, tu as regardé. Te voilà. Il est chaud. [pause]</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr"/>
@@ -1629,7 +1643,7 @@
         </is>
       </c>
       <c r="Y4" s="2" t="n">
-        <v>118</v>
+        <v>140</v>
       </c>
       <c r="Z4" s="2" t="inlineStr">
         <is>
@@ -1637,10 +1651,10 @@
         </is>
       </c>
       <c r="AA4" s="2" t="n">
-        <v>0.86</v>
+        <v>0.97</v>
       </c>
       <c r="AB4" s="2" t="n">
-        <v>1.22</v>
+        <v>1.14</v>
       </c>
       <c r="AC4" s="2" t="inlineStr">
         <is>
@@ -1663,30 +1677,30 @@
       </c>
       <c r="AH4" s="2" t="inlineStr">
         <is>
-          <t>une</t>
+          <t>éclat de marche</t>
         </is>
       </c>
       <c r="AI4" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ4" s="2" t="n">
-        <v>450</v>
+        <v>560</v>
       </c>
       <c r="AK4" s="2" t="n">
-        <v>380</v>
+        <v>270</v>
       </c>
       <c r="AL4" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>bright</t>
         </is>
       </c>
       <c r="AM4" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="AN4" s="2" t="n">
-        <v>0.333</v>
+        <v>0.35</v>
       </c>
       <c r="AO4" s="2" t="inlineStr"/>
       <c r="AP4" s="2" t="inlineStr">
@@ -1695,10 +1709,10 @@
         </is>
       </c>
       <c r="AQ4" s="2" t="n">
-        <v>0.86</v>
+        <v>0.97</v>
       </c>
       <c r="AR4" s="2" t="n">
-        <v>0.86</v>
+        <v>0.97</v>
       </c>
       <c r="AS4" s="2" t="n">
         <v>100</v>
@@ -1707,32 +1721,56 @@
         <v>50</v>
       </c>
       <c r="AU4" s="2" t="n">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="AV4" s="2" t="inlineStr">
         <is>
-          <t>confirmation ; le moteur peut dire engine_ok/near avant ce chunk</t>
+          <t>arc=résolution; intention=faire_vivre_le_geste; emotion=concentration puis fierté_calme; intensite=2; destinataire=enfant; sous_texte=il_refuse_de_foncer_retrouve_l_eclat; tempo=naturel; sourire=léger; respiration=relâchée</t>
         </is>
       </c>
       <c r="AW4" t="inlineStr">
         <is>
-          <t>narrateur|Le pull jaune est près du lit.
-narrateur|Nino enfile le pull.
+          <t>narrateur|Nino revient vers le lit.
+narrateur|Ses pieds touchent le tapis.
+narrateur|Le pull jaune est près du lit.
+enfant-m|Toi d'abord.
+narrateur|Il enfile le pull.
 narrateur|Le pull est doux sur les bras.
+narrateur|Le pyjama reste en dessous, chaud.
 enfant-m|C'est fait.
-maman|Ensuite, les marches.
-narrateur|Nino pose la main sur la rampe.
-maman|Une marche, puis l'autre.
+maman|Tu vas vers les marches ?
 enfant-m|Oui, maman.
-narrateur|Les marches sentent le bois.
+narrateur|Nino s'arrête devant la première marche.
+narrateur|L'éclat de marche brille, petit.
+enfant-m|Je te vois.
+narrateur|Sa main trouve la rampe.
+narrateur|La rampe est ronde, un peu froide.
+narrateur|Une marche, sous le pied.
+narrateur|Puis une autre.
+enfant-m|Je regarde.
+narrateur|Au milieu, une chaussette traîne.
+enfant-m|Je la pousse.
+narrateur|Nino lève le pied, trop vite.
+narrateur|Puis il s'arrête.
+enfant-m|Attends.
+narrateur|Nino refuse de foncer.
+narrateur|Il ramasse la chaussette.
+narrateur|Sous le tissu, l'éclat de marche brille.
+enfant-m|Comme en haut !
+papa|Tu le vois, toi ?
+enfant-m|Oui, près du bois.
+narrateur|Nino glisse la chaussette dans sa main.
+narrateur|Il descend, sans sauter.
 narrateur|La cuisine est chaude.
 narrateur|Le pain est sur la planche.
-narrateur|La croûte craque un peu.
-papa|Tu t'assois ?
-narrateur|Nino s'assoit à table.
-maman|Un peu de beurre ?
-enfant-m|Oui, un peu.
-papa|Merci, Nino.</t>
+papa|Merci, tu as regardé.
+maman|Te voilà.
+enfant-m|Il est chaud.</t>
+        </is>
+      </c>
+      <c r="AX4" t="inlineStr">
+        <is>
+          <t>pull,marches</t>
         </is>
       </c>
     </row>
@@ -1759,17 +1797,17 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>Nino mord la croûte. Le pain est tiède. Le beurre fond un peu. C'est bon. Tu as une miette ici. Papa montre le menton. Je l'essuie. Ensuite, le sac. Le sac vert est près du banc. Nino glisse le doudou. Le tissu est encore chaud. Le pain est tout près ? Oui, papa. Nino met ses chaussures. Le pied gauche d'abord ? Oui. Maman ouvre la porte. L'air sent encore le pain. Ça sent bon. Oui. Nino sent ses doigts. Ils sentent encore le beurre. Le pain est venu jusqu'à toi. Une miette dore encore sur la planche. La rampe de bois reste tiède. Tu as pris le temps ? Oui, une chose, puis l'autre.</t>
+          <t>Tu t'assois ? Nino s'assoit à table. Un peu de beurre ? Oui, un peu. Le beurre fond sur la croûte. Nino mord la croûte. Le pain est tiède. C'est bon. Tu as une miette ici. Papa montre le menton. Je l'essuie. On le mange ici. Oui, ici. Nino lève les yeux vers l'escalier. Sur la première marche, l'éclat de marche brille. Il est là, papa. Comme tout à l'heure. La chaleur touche les joues de Nino. On est bien, ici. Le pain est venu. La rampe de bois reste tiède. Nino sent le beurre sur ses doigts.</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>Nino mord la croûte. Le pain est tiède. Le beurre fond un peu. C'est bon. Tu as une miette ici. Papa montre le menton. Je l'essuie. Ensuite, le sac. Le sac vert est près du banc. Nino glisse le doudou. Le tissu est encore chaud. Le pain est tout près ? Oui, papa. Nino met ses chaussures. Le pied gauche d'abord ? Oui. Maman ouvre la porte. L'air sent encore le pain. Ça sent bon. Oui. Nino sent ses doigts. Ils sentent encore le beurre. Le pain est venu jusqu'à toi. Une miette dore encore sur la planche. La rampe de bois reste tiède. Tu as pris le temps ? Oui, une chose, puis l'autre.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Tu t'assois ? Nino s'assoit à table. Un peu de beurre ? Oui, un peu. Le beurre fond sur la croûte. Nino mord la croûte. Le &lt;emphasis level="moderate"&gt;pain&lt;/emphasis&gt; est tiède. C'est bon. Tu as une miette ici. Papa montre le menton. Je l'essuie. On le mange ici. Oui, ici. Nino lève les yeux vers l'escalier. Sur la première marche, l'éclat de marche brille. Il est là, papa. Comme tout à l'heure. La chaleur touche les joues de Nino. On est bien, ici. Le pain est venu. La rampe de bois reste tiède. Nino sent le beurre sur ses doigts.&lt;/prosody&gt;&lt;break time="420ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;Ilyes met les chaussures. Maman ouvre la porte. L'air sent le matin.&lt;/slow&gt; [pause]</t>
+          <t>Tu t'assois ? Nino s'assoit à table. Un peu de beurre ? Oui, un peu. Le beurre fond sur la croûte. Nino mord la croûte. Le &lt;emphasis&gt;pain&lt;/emphasis&gt; est tiède. C'est bon. Tu as une miette ici. Papa montre le menton. Je l'essuie. On le mange ici. Oui, ici. Nino lève les yeux vers l'escalier. Sur la première marche, l'éclat de marche brille. Il est là, papa. Comme tout à l'heure. La chaleur touche les joues de Nino. On est bien, ici. Le pain est venu. La rampe de bois reste tiède. Nino sent le beurre sur ses doigts. [pause]</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr"/>
@@ -1816,7 +1854,7 @@
         </is>
       </c>
       <c r="Y5" s="2" t="n">
-        <v>118</v>
+        <v>146</v>
       </c>
       <c r="Z5" s="2" t="inlineStr">
         <is>
@@ -1824,10 +1862,10 @@
         </is>
       </c>
       <c r="AA5" s="2" t="n">
-        <v>0.86</v>
+        <v>1</v>
       </c>
       <c r="AB5" s="2" t="n">
-        <v>1.22</v>
+        <v>1.1</v>
       </c>
       <c r="AC5" s="2" t="inlineStr">
         <is>
@@ -1848,28 +1886,32 @@
       <c r="AG5" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="AH5" s="2" t="inlineStr"/>
+      <c r="AH5" s="2" t="inlineStr">
+        <is>
+          <t>pain</t>
+        </is>
+      </c>
       <c r="AI5" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ5" s="2" t="n">
-        <v>450</v>
+        <v>420</v>
       </c>
       <c r="AK5" s="2" t="n">
-        <v>380</v>
+        <v>250</v>
       </c>
       <c r="AL5" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>lively</t>
         </is>
       </c>
       <c r="AM5" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>dynamic</t>
         </is>
       </c>
       <c r="AN5" s="2" t="n">
-        <v>0.333</v>
+        <v>0.37</v>
       </c>
       <c r="AO5" s="2" t="inlineStr"/>
       <c r="AP5" s="2" t="inlineStr">
@@ -1878,10 +1920,10 @@
         </is>
       </c>
       <c r="AQ5" s="2" t="n">
-        <v>0.86</v>
+        <v>1</v>
       </c>
       <c r="AR5" s="2" t="n">
-        <v>0.86</v>
+        <v>1</v>
       </c>
       <c r="AS5" s="2" t="n">
         <v>100</v>
@@ -1890,43 +1932,42 @@
         <v>50</v>
       </c>
       <c r="AU5" s="2" t="n">
-        <v>12</v>
-      </c>
-      <c r="AV5" s="2" t="inlineStr"/>
+        <v>8</v>
+      </c>
+      <c r="AV5" s="2" t="inlineStr">
+        <is>
+          <t>arc=action; intention=refermer_le_désir; emotion=fierté_calme et chaleur; intensite=2; destinataire=enfant; sous_texte=le_pain_arrive_jusqu_a_lui; tempo=vif puis posé; sourire=léger; respiration=courte</t>
+        </is>
+      </c>
       <c r="AW5" t="inlineStr">
         <is>
-          <t>narrateur|Nino mord la croûte.
+          <t>papa|Tu t'assois ?
+narrateur|Nino s'assoit à table.
+maman|Un peu de beurre ?
+enfant-m|Oui, un peu.
+narrateur|Le beurre fond sur la croûte.
+narrateur|Nino mord la croûte.
 narrateur|Le pain est tiède.
-narrateur|Le beurre fond un peu.
 enfant-m|C'est bon.
 papa|Tu as une miette ici.
 narrateur|Papa montre le menton.
 enfant-m|Je l'essuie.
-maman|Ensuite, le sac.
-narrateur|Le sac vert est près du banc.
-narrateur|Nino glisse le doudou.
-narrateur|Le tissu est encore chaud.
-papa|Le pain est tout près ?
-enfant-m|Oui, papa.
-narrateur|Nino met ses chaussures.
-papa|Le pied gauche d'abord ?
-enfant-m|Oui.
-narrateur|Maman ouvre la porte.
-narrateur|L'air sent encore le pain.
-enfant-m|Ça sent bon.
-maman|Oui.
-narrateur|Nino sent ses doigts.
-narrateur|Ils sentent encore le beurre.
-papa|Le pain est venu jusqu'à toi.
-narrateur|Une miette dore encore sur la planche.
+maman|On le mange ici.
+enfant-m|Oui, ici.
+narrateur|Nino lève les yeux vers l'escalier.
+narrateur|Sur la première marche, l'éclat de marche brille.
+enfant-m|Il est là, papa.
+papa|Comme tout à l'heure.
+narrateur|La chaleur touche les joues de Nino.
+maman|On est bien, ici.
+enfant-m|Le pain est venu.
 narrateur|La rampe de bois reste tiède.
-maman|Tu as pris le temps ?
-enfant-m|Oui, une chose, puis l'autre.</t>
+narrateur|Nino sent le beurre sur ses doigts.</t>
         </is>
       </c>
       <c r="AX5" t="inlineStr">
         <is>
-          <t>porte</t>
+          <t>pain,beurre</t>
         </is>
       </c>
     </row>
@@ -1953,17 +1994,17 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>Le pain était chaud. Tu es venu jusqu'à lui. Une chose, puis la suivante. Une petite vapeur flotte encore. Bravo, Nino. La croûte tiède reste sur sa langue.</t>
+          <t>Le pain était chaud. Tu es venu jusqu'à lui. Une petite vapeur flotte, blanche. Nino sent le beurre sur sa langue. Sur la croûte, l'éclat de marche garde une trace.</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>Le pain était chaud. Tu es venu jusqu'à lui. Une chose, puis la suivante. Une petite vapeur flotte encore. Bravo, Nino. La croûte tiède reste sur sa langue.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Le pain était chaud. Tu es venu jusqu'à lui. Une petite vapeur flotte, blanche. Nino sent le beurre sur sa langue. Sur la croûte, l'&lt;emphasis level="moderate"&gt;éclat de marche&lt;/emphasis&gt; garde une trace.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>&lt;lower-pitch&gt;&lt;soft&gt;&lt;slow&gt;L'histoire est finie.&lt;/slow&gt;&lt;/soft&gt;&lt;/lower-pitch&gt; [pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Le pain était chaud. Tu es venu jusqu'à lui. Une petite vapeur flotte, blanche. Nino sent le beurre sur sa langue. Sur la croûte, l'&lt;emphasis&gt;éclat de marche&lt;/emphasis&gt; garde une trace.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr"/>
@@ -2010,18 +2051,18 @@
         </is>
       </c>
       <c r="Y6" s="2" t="n">
-        <v>106</v>
+        <v>118</v>
       </c>
       <c r="Z6" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>slow</t>
         </is>
       </c>
       <c r="AA6" s="2" t="n">
-        <v>0.82</v>
+        <v>0.85</v>
       </c>
       <c r="AB6" s="2" t="n">
-        <v>1.22</v>
+        <v>1.28</v>
       </c>
       <c r="AC6" s="2" t="inlineStr">
         <is>
@@ -2030,12 +2071,12 @@
       </c>
       <c r="AD6" s="2" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>-2st</t>
         </is>
       </c>
       <c r="AE6" s="2" t="inlineStr">
         <is>
-          <t>lower-pitch</t>
+          <t>low-pitch</t>
         </is>
       </c>
       <c r="AF6" s="2" t="inlineStr">
@@ -2044,17 +2085,21 @@
         </is>
       </c>
       <c r="AG6" s="2" t="n">
-        <v>-2</v>
-      </c>
-      <c r="AH6" s="2" t="inlineStr"/>
+        <v>-3</v>
+      </c>
+      <c r="AH6" s="2" t="inlineStr">
+        <is>
+          <t>éclat de marche</t>
+        </is>
+      </c>
       <c r="AI6" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ6" s="2" t="n">
-        <v>600</v>
+        <v>900</v>
       </c>
       <c r="AK6" s="2" t="n">
-        <v>380</v>
+        <v>340</v>
       </c>
       <c r="AL6" s="2" t="inlineStr">
         <is>
@@ -2063,11 +2108,11 @@
       </c>
       <c r="AM6" s="2" t="inlineStr">
         <is>
-          <t>fall</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="AN6" s="2" t="n">
-        <v>0.333</v>
+        <v>0.31</v>
       </c>
       <c r="AO6" s="2" t="inlineStr"/>
       <c r="AP6" s="2" t="inlineStr">
@@ -2076,29 +2121,37 @@
         </is>
       </c>
       <c r="AQ6" s="2" t="n">
-        <v>0.82</v>
+        <v>0.85</v>
       </c>
       <c r="AR6" s="2" t="n">
-        <v>0.82</v>
+        <v>0.85</v>
       </c>
       <c r="AS6" s="2" t="n">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="AT6" s="2" t="n">
-        <v>35</v>
+        <v>42</v>
       </c>
       <c r="AU6" s="2" t="n">
         <v>12</v>
       </c>
-      <c r="AV6" s="2" t="inlineStr"/>
+      <c r="AV6" s="2" t="inlineStr">
+        <is>
+          <t>arc=retour; intention=refermer; emotion=tendresse et fierté_calme; intensite=1; destinataire=enfant; sous_texte=l_eclat_de_la_marche_est_sur_la_croute; tempo=posé; sourire=léger; respiration=ample</t>
+        </is>
+      </c>
       <c r="AW6" t="inlineStr">
         <is>
           <t>enfant-m|Le pain était chaud.
 maman|Tu es venu jusqu'à lui.
-papa|Une chose, puis la suivante.
-narrateur|Une petite vapeur flotte encore.
-maman|Bravo, Nino.
-narrateur|La croûte tiède reste sur sa langue.</t>
+narrateur|Une petite vapeur flotte, blanche.
+narrateur|Nino sent le beurre sur sa langue.
+narrateur|Sur la croûte, l'éclat de marche garde une trace.</t>
+        </is>
+      </c>
+      <c r="AX6" t="inlineStr">
+        <is>
+          <t>pain</t>
         </is>
       </c>
     </row>
@@ -2119,7 +2172,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A14"/>
+  <dimension ref="A1:A15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -2218,6 +2271,13 @@
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
+        <is>
+          <t>F-NAR-008 récit, pas une leçon en puces</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
         <is>
           <t>F-NAR-008 récit, pas une leçon en puces</t>
         </is>

</xml_diff>